<commit_message>
Update: Optimized PPC conversion funnel logic and fixed CVR calculation
</commit_message>
<xml_diff>
--- a/C_mass_sop_factory/data/output/Bulk_Create_250TH_250YEARSOFFREEDOM_JAR.xlsx
+++ b/C_mass_sop_factory/data/output/Bulk_Create_250TH_250YEARSOFFREEDOM_JAR.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="928" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="878" uniqueCount="70">
   <si>
     <t>Product</t>
   </si>
@@ -121,88 +121,85 @@
     <t>Create</t>
   </si>
   <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_exact_4th of july decorations_30TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_exact_fourth of july decorations_30TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_exact_patriotic decorations_30TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_exact_4th of july cards_30TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_exact_america anniversary gifts_30TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_exact_patriotic affirmation jar_30TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_phrase_4th of july decorations_30TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_phrase_fourth of july decorations_30TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_phrase_patriotic decorations_30TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_phrase_4th of july cards_30TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_phrase_america anniversary gifts_30TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_phrase_patriotic affirmation jar_30TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_broad_4th of july decorations_20TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_broad_fourth of july decorations_20TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_broad_patriotic decorations_20TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_broad_4th of july cards_20TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_broad_america anniversary gifts_20TRP</t>
-  </si>
-  <si>
-    <t>250TH_250YEARSOFFREEDOM_JAR_KT_broad_patriotic affirmation jar_20TRP</t>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_exact_fourth_of_july_decorations_30TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_exact_patriotic_decorations_30TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_exact_4th_of_july_cards_30TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_exact_america_anniversary_gifts_30TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_exact_patriotic_affirmation_jar_30TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_phrase_4th_of_july_decorations_30TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_phrase_fourth_of_july_decorations_30TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_phrase_patriotic_decorations_30TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_phrase_4th_of_july_cards_30TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_phrase_america_anniversary_gifts_30TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_phrase_patriotic_affirmation_jar_30TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_broad_4th_of_july_decorations_20TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_broad_fourth_of_july_decorations_20TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_broad_patriotic_decorations_20TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_broad_4th_of_july_cards_20TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_broad_america_anniversary_gifts_20TRP</t>
+  </si>
+  <si>
+    <t>250TH_250YEARSOFFREEDOM_JAR_KT_broad_patriotic_affirmation_jar_20TRP</t>
   </si>
   <si>
     <t>128613535409943</t>
   </si>
   <si>
+    <t>fourth of july decorations</t>
+  </si>
+  <si>
+    <t>patriotic decorations</t>
+  </si>
+  <si>
+    <t>4th of july cards</t>
+  </si>
+  <si>
+    <t>america anniversary gifts</t>
+  </si>
+  <si>
+    <t>patriotic affirmation jar</t>
+  </si>
+  <si>
     <t>4th of july decorations</t>
   </si>
   <si>
-    <t>fourth of july decorations</t>
-  </si>
-  <si>
-    <t>patriotic decorations</t>
-  </si>
-  <si>
-    <t>4th of july cards</t>
-  </si>
-  <si>
-    <t>america anniversary gifts</t>
-  </si>
-  <si>
-    <t>patriotic affirmation jar</t>
-  </si>
-  <si>
-    <t>20260418</t>
-  </si>
-  <si>
-    <t>MANUAL</t>
-  </si>
-  <si>
-    <t>enabled</t>
+    <t>20260423</t>
+  </si>
+  <si>
+    <t>Manual</t>
+  </si>
+  <si>
+    <t>Enabled</t>
   </si>
   <si>
     <t>250TH_250YEARSOFFREEDOM_JAR</t>
@@ -220,13 +217,13 @@
     <t>Dynamic bids - down only</t>
   </si>
   <si>
-    <t>placement top</t>
-  </si>
-  <si>
-    <t>placementProductPage</t>
-  </si>
-  <si>
-    <t>placementRestOfSearch</t>
+    <t>Placement Top</t>
+  </si>
+  <si>
+    <t>Placement Product Page</t>
+  </si>
+  <si>
+    <t>Placement Rest Of Search</t>
   </si>
 </sst>
 </file>
@@ -588,7 +585,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB127"/>
+  <dimension ref="A1:AB120"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="28" width="20.7109375" style="1" customWidth="1"/>
@@ -694,25 +691,25 @@
         <v>35</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>35</v>
       </c>
       <c r="L2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N2" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N2" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O2" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P2" s="1">
         <v>5</v>
       </c>
       <c r="Y2" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:28">
@@ -729,10 +726,10 @@
         <v>35</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA3" s="1">
         <v>30</v>
@@ -752,10 +749,10 @@
         <v>35</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA4" s="1">
         <v>30</v>
@@ -775,10 +772,10 @@
         <v>35</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA5" s="1">
         <v>30</v>
@@ -801,10 +798,10 @@
         <v>35</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U6" s="1">
         <v>0.6</v>
@@ -827,10 +824,10 @@
         <v>35</v>
       </c>
       <c r="O7" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q7" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q7" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:28">
@@ -850,16 +847,16 @@
         <v>35</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V8" s="1">
         <v>0.6</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="X8" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:28">
@@ -876,25 +873,25 @@
         <v>36</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>36</v>
       </c>
       <c r="L9" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N9" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N9" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O9" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P9" s="1">
         <v>5</v>
       </c>
       <c r="Y9" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:28">
@@ -911,10 +908,10 @@
         <v>36</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z10" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA10" s="1">
         <v>30</v>
@@ -934,10 +931,10 @@
         <v>36</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z11" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA11" s="1">
         <v>30</v>
@@ -957,10 +954,10 @@
         <v>36</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z12" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA12" s="1">
         <v>30</v>
@@ -983,10 +980,10 @@
         <v>36</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U13" s="1">
         <v>0.6</v>
@@ -1009,10 +1006,10 @@
         <v>36</v>
       </c>
       <c r="O14" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q14" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q14" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:28">
@@ -1032,16 +1029,16 @@
         <v>36</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V15" s="1">
         <v>0.6</v>
       </c>
       <c r="W15" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="X15" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:28">
@@ -1058,25 +1055,25 @@
         <v>37</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>37</v>
       </c>
       <c r="L16" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N16" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N16" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O16" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P16" s="1">
         <v>5</v>
       </c>
       <c r="Y16" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:27">
@@ -1093,10 +1090,10 @@
         <v>37</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z17" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA17" s="1">
         <v>30</v>
@@ -1116,10 +1113,10 @@
         <v>37</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z18" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA18" s="1">
         <v>30</v>
@@ -1139,10 +1136,10 @@
         <v>37</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z19" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA19" s="1">
         <v>30</v>
@@ -1165,10 +1162,10 @@
         <v>37</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U20" s="1">
         <v>0.6</v>
@@ -1191,10 +1188,10 @@
         <v>37</v>
       </c>
       <c r="O21" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q21" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q21" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:27">
@@ -1214,16 +1211,16 @@
         <v>37</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V22" s="1">
         <v>0.6</v>
       </c>
       <c r="W22" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="X22" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:27">
@@ -1240,25 +1237,25 @@
         <v>38</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J23" s="1" t="s">
         <v>38</v>
       </c>
       <c r="L23" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N23" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N23" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O23" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P23" s="1">
         <v>5</v>
       </c>
       <c r="Y23" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:27">
@@ -1275,10 +1272,10 @@
         <v>38</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z24" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA24" s="1">
         <v>30</v>
@@ -1298,10 +1295,10 @@
         <v>38</v>
       </c>
       <c r="O25" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z25" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA25" s="1">
         <v>30</v>
@@ -1321,10 +1318,10 @@
         <v>38</v>
       </c>
       <c r="O26" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z26" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA26" s="1">
         <v>30</v>
@@ -1347,10 +1344,10 @@
         <v>38</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="O27" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U27" s="1">
         <v>0.6</v>
@@ -1373,10 +1370,10 @@
         <v>38</v>
       </c>
       <c r="O28" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q28" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q28" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="29" spans="1:27">
@@ -1396,16 +1393,16 @@
         <v>38</v>
       </c>
       <c r="O29" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V29" s="1">
         <v>0.6</v>
       </c>
       <c r="W29" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="X29" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="30" spans="1:27">
@@ -1422,25 +1419,25 @@
         <v>39</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J30" s="1" t="s">
         <v>39</v>
       </c>
       <c r="L30" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N30" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N30" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O30" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P30" s="1">
         <v>5</v>
       </c>
       <c r="Y30" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="31" spans="1:27">
@@ -1457,10 +1454,10 @@
         <v>39</v>
       </c>
       <c r="O31" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z31" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA31" s="1">
         <v>30</v>
@@ -1480,10 +1477,10 @@
         <v>39</v>
       </c>
       <c r="O32" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z32" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA32" s="1">
         <v>30</v>
@@ -1503,10 +1500,10 @@
         <v>39</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z33" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA33" s="1">
         <v>30</v>
@@ -1529,10 +1526,10 @@
         <v>39</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="O34" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U34" s="1">
         <v>0.6</v>
@@ -1555,10 +1552,10 @@
         <v>39</v>
       </c>
       <c r="O35" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q35" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q35" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="36" spans="1:27">
@@ -1578,16 +1575,16 @@
         <v>39</v>
       </c>
       <c r="O36" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V36" s="1">
         <v>0.6</v>
       </c>
       <c r="W36" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="X36" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="37" spans="1:27">
@@ -1604,25 +1601,25 @@
         <v>40</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J37" s="1" t="s">
         <v>40</v>
       </c>
       <c r="L37" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N37" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N37" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O37" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P37" s="1">
         <v>5</v>
       </c>
       <c r="Y37" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="38" spans="1:27">
@@ -1639,10 +1636,10 @@
         <v>40</v>
       </c>
       <c r="O38" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z38" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA38" s="1">
         <v>30</v>
@@ -1662,10 +1659,10 @@
         <v>40</v>
       </c>
       <c r="O39" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z39" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA39" s="1">
         <v>30</v>
@@ -1685,10 +1682,10 @@
         <v>40</v>
       </c>
       <c r="O40" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z40" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA40" s="1">
         <v>30</v>
@@ -1711,13 +1708,13 @@
         <v>40</v>
       </c>
       <c r="K41" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O41" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U41" s="1">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="42" spans="1:27">
@@ -1737,10 +1734,10 @@
         <v>40</v>
       </c>
       <c r="O42" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q42" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q42" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="43" spans="1:27">
@@ -1760,13 +1757,13 @@
         <v>40</v>
       </c>
       <c r="O43" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V43" s="1">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="W43" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="X43" s="1" t="s">
         <v>64</v>
@@ -1786,25 +1783,25 @@
         <v>41</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J44" s="1" t="s">
         <v>41</v>
       </c>
       <c r="L44" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N44" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N44" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O44" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P44" s="1">
         <v>5</v>
       </c>
       <c r="Y44" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="45" spans="1:27">
@@ -1821,10 +1818,10 @@
         <v>41</v>
       </c>
       <c r="O45" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z45" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA45" s="1">
         <v>30</v>
@@ -1844,10 +1841,10 @@
         <v>41</v>
       </c>
       <c r="O46" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z46" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA46" s="1">
         <v>30</v>
@@ -1867,10 +1864,10 @@
         <v>41</v>
       </c>
       <c r="O47" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z47" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA47" s="1">
         <v>30</v>
@@ -1893,10 +1890,10 @@
         <v>41</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="O48" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U48" s="1">
         <v>0.4</v>
@@ -1919,10 +1916,10 @@
         <v>41</v>
       </c>
       <c r="O49" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q49" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q49" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="50" spans="1:27">
@@ -1942,16 +1939,16 @@
         <v>41</v>
       </c>
       <c r="O50" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V50" s="1">
         <v>0.4</v>
       </c>
       <c r="W50" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="X50" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="51" spans="1:27">
@@ -1968,25 +1965,25 @@
         <v>42</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J51" s="1" t="s">
         <v>42</v>
       </c>
       <c r="L51" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N51" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N51" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O51" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P51" s="1">
         <v>5</v>
       </c>
       <c r="Y51" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="52" spans="1:27">
@@ -2003,10 +2000,10 @@
         <v>42</v>
       </c>
       <c r="O52" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z52" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA52" s="1">
         <v>30</v>
@@ -2026,10 +2023,10 @@
         <v>42</v>
       </c>
       <c r="O53" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z53" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA53" s="1">
         <v>30</v>
@@ -2049,10 +2046,10 @@
         <v>42</v>
       </c>
       <c r="O54" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z54" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA54" s="1">
         <v>30</v>
@@ -2075,10 +2072,10 @@
         <v>42</v>
       </c>
       <c r="K55" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O55" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U55" s="1">
         <v>0.4</v>
@@ -2101,10 +2098,10 @@
         <v>42</v>
       </c>
       <c r="O56" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q56" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q56" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="57" spans="1:27">
@@ -2124,16 +2121,16 @@
         <v>42</v>
       </c>
       <c r="O57" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V57" s="1">
         <v>0.4</v>
       </c>
       <c r="W57" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="X57" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="58" spans="1:27">
@@ -2150,25 +2147,25 @@
         <v>43</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J58" s="1" t="s">
         <v>43</v>
       </c>
       <c r="L58" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N58" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N58" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O58" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P58" s="1">
         <v>5</v>
       </c>
       <c r="Y58" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="59" spans="1:27">
@@ -2185,10 +2182,10 @@
         <v>43</v>
       </c>
       <c r="O59" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z59" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA59" s="1">
         <v>30</v>
@@ -2208,10 +2205,10 @@
         <v>43</v>
       </c>
       <c r="O60" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z60" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA60" s="1">
         <v>30</v>
@@ -2231,10 +2228,10 @@
         <v>43</v>
       </c>
       <c r="O61" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z61" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA61" s="1">
         <v>30</v>
@@ -2257,10 +2254,10 @@
         <v>43</v>
       </c>
       <c r="K62" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="O62" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U62" s="1">
         <v>0.4</v>
@@ -2283,10 +2280,10 @@
         <v>43</v>
       </c>
       <c r="O63" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q63" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q63" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="64" spans="1:27">
@@ -2306,16 +2303,16 @@
         <v>43</v>
       </c>
       <c r="O64" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V64" s="1">
         <v>0.4</v>
       </c>
       <c r="W64" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="X64" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="65" spans="1:27">
@@ -2332,25 +2329,25 @@
         <v>44</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J65" s="1" t="s">
         <v>44</v>
       </c>
       <c r="L65" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N65" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N65" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O65" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P65" s="1">
         <v>5</v>
       </c>
       <c r="Y65" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="66" spans="1:27">
@@ -2367,10 +2364,10 @@
         <v>44</v>
       </c>
       <c r="O66" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z66" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA66" s="1">
         <v>30</v>
@@ -2390,10 +2387,10 @@
         <v>44</v>
       </c>
       <c r="O67" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z67" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA67" s="1">
         <v>30</v>
@@ -2413,10 +2410,10 @@
         <v>44</v>
       </c>
       <c r="O68" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z68" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA68" s="1">
         <v>30</v>
@@ -2439,10 +2436,10 @@
         <v>44</v>
       </c>
       <c r="K69" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="O69" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U69" s="1">
         <v>0.4</v>
@@ -2465,10 +2462,10 @@
         <v>44</v>
       </c>
       <c r="O70" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q70" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q70" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="71" spans="1:27">
@@ -2488,16 +2485,16 @@
         <v>44</v>
       </c>
       <c r="O71" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V71" s="1">
         <v>0.4</v>
       </c>
       <c r="W71" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="X71" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="72" spans="1:27">
@@ -2514,25 +2511,25 @@
         <v>45</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J72" s="1" t="s">
         <v>45</v>
       </c>
       <c r="L72" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N72" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N72" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O72" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P72" s="1">
         <v>5</v>
       </c>
       <c r="Y72" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="73" spans="1:27">
@@ -2549,10 +2546,10 @@
         <v>45</v>
       </c>
       <c r="O73" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z73" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA73" s="1">
         <v>30</v>
@@ -2572,10 +2569,10 @@
         <v>45</v>
       </c>
       <c r="O74" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z74" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA74" s="1">
         <v>30</v>
@@ -2595,10 +2592,10 @@
         <v>45</v>
       </c>
       <c r="O75" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z75" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA75" s="1">
         <v>30</v>
@@ -2621,10 +2618,10 @@
         <v>45</v>
       </c>
       <c r="K76" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="O76" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U76" s="1">
         <v>0.4</v>
@@ -2647,10 +2644,10 @@
         <v>45</v>
       </c>
       <c r="O77" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q77" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q77" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="78" spans="1:27">
@@ -2670,16 +2667,16 @@
         <v>45</v>
       </c>
       <c r="O78" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V78" s="1">
         <v>0.4</v>
       </c>
       <c r="W78" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="X78" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="79" spans="1:27">
@@ -2696,25 +2693,25 @@
         <v>46</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J79" s="1" t="s">
         <v>46</v>
       </c>
       <c r="L79" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N79" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N79" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O79" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P79" s="1">
         <v>5</v>
       </c>
       <c r="Y79" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="80" spans="1:27">
@@ -2731,13 +2728,13 @@
         <v>46</v>
       </c>
       <c r="O80" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z80" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA80" s="1">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="81" spans="1:27">
@@ -2754,13 +2751,13 @@
         <v>46</v>
       </c>
       <c r="O81" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z81" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA81" s="1">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="82" spans="1:27">
@@ -2777,13 +2774,13 @@
         <v>46</v>
       </c>
       <c r="O82" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z82" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA82" s="1">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="83" spans="1:27">
@@ -2803,13 +2800,13 @@
         <v>46</v>
       </c>
       <c r="K83" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O83" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U83" s="1">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="84" spans="1:27">
@@ -2829,10 +2826,10 @@
         <v>46</v>
       </c>
       <c r="O84" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q84" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q84" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="85" spans="1:27">
@@ -2852,13 +2849,13 @@
         <v>46</v>
       </c>
       <c r="O85" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V85" s="1">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="W85" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="X85" s="1" t="s">
         <v>65</v>
@@ -2878,25 +2875,25 @@
         <v>47</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J86" s="1" t="s">
         <v>47</v>
       </c>
       <c r="L86" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N86" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N86" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O86" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P86" s="1">
         <v>5</v>
       </c>
       <c r="Y86" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="87" spans="1:27">
@@ -2913,10 +2910,10 @@
         <v>47</v>
       </c>
       <c r="O87" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z87" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA87" s="1">
         <v>20</v>
@@ -2936,10 +2933,10 @@
         <v>47</v>
       </c>
       <c r="O88" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z88" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA88" s="1">
         <v>20</v>
@@ -2959,10 +2956,10 @@
         <v>47</v>
       </c>
       <c r="O89" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z89" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA89" s="1">
         <v>20</v>
@@ -2985,10 +2982,10 @@
         <v>47</v>
       </c>
       <c r="K90" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="O90" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U90" s="1">
         <v>0.35</v>
@@ -3011,10 +3008,10 @@
         <v>47</v>
       </c>
       <c r="O91" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q91" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q91" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="92" spans="1:27">
@@ -3034,16 +3031,16 @@
         <v>47</v>
       </c>
       <c r="O92" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V92" s="1">
         <v>0.35</v>
       </c>
       <c r="W92" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="X92" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="93" spans="1:27">
@@ -3060,25 +3057,25 @@
         <v>48</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J93" s="1" t="s">
         <v>48</v>
       </c>
       <c r="L93" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N93" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N93" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O93" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P93" s="1">
         <v>5</v>
       </c>
       <c r="Y93" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="94" spans="1:27">
@@ -3095,10 +3092,10 @@
         <v>48</v>
       </c>
       <c r="O94" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z94" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA94" s="1">
         <v>20</v>
@@ -3118,10 +3115,10 @@
         <v>48</v>
       </c>
       <c r="O95" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z95" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA95" s="1">
         <v>20</v>
@@ -3141,10 +3138,10 @@
         <v>48</v>
       </c>
       <c r="O96" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z96" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA96" s="1">
         <v>20</v>
@@ -3167,10 +3164,10 @@
         <v>48</v>
       </c>
       <c r="K97" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O97" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U97" s="1">
         <v>0.35</v>
@@ -3193,10 +3190,10 @@
         <v>48</v>
       </c>
       <c r="O98" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q98" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q98" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="99" spans="1:27">
@@ -3216,16 +3213,16 @@
         <v>48</v>
       </c>
       <c r="O99" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V99" s="1">
         <v>0.35</v>
       </c>
       <c r="W99" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="X99" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="100" spans="1:27">
@@ -3242,25 +3239,25 @@
         <v>49</v>
       </c>
       <c r="F100" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J100" s="1" t="s">
         <v>49</v>
       </c>
       <c r="L100" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N100" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N100" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O100" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P100" s="1">
         <v>5</v>
       </c>
       <c r="Y100" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="101" spans="1:27">
@@ -3277,10 +3274,10 @@
         <v>49</v>
       </c>
       <c r="O101" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z101" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA101" s="1">
         <v>20</v>
@@ -3300,10 +3297,10 @@
         <v>49</v>
       </c>
       <c r="O102" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z102" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA102" s="1">
         <v>20</v>
@@ -3323,10 +3320,10 @@
         <v>49</v>
       </c>
       <c r="O103" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z103" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA103" s="1">
         <v>20</v>
@@ -3349,10 +3346,10 @@
         <v>49</v>
       </c>
       <c r="K104" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="O104" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U104" s="1">
         <v>0.35</v>
@@ -3375,10 +3372,10 @@
         <v>49</v>
       </c>
       <c r="O105" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q105" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q105" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="106" spans="1:27">
@@ -3398,16 +3395,16 @@
         <v>49</v>
       </c>
       <c r="O106" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V106" s="1">
         <v>0.35</v>
       </c>
       <c r="W106" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="X106" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="107" spans="1:27">
@@ -3424,25 +3421,25 @@
         <v>50</v>
       </c>
       <c r="F107" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J107" s="1" t="s">
         <v>50</v>
       </c>
       <c r="L107" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N107" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N107" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O107" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P107" s="1">
         <v>5</v>
       </c>
       <c r="Y107" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="108" spans="1:27">
@@ -3459,10 +3456,10 @@
         <v>50</v>
       </c>
       <c r="O108" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z108" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA108" s="1">
         <v>20</v>
@@ -3482,10 +3479,10 @@
         <v>50</v>
       </c>
       <c r="O109" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z109" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA109" s="1">
         <v>20</v>
@@ -3505,10 +3502,10 @@
         <v>50</v>
       </c>
       <c r="O110" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z110" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA110" s="1">
         <v>20</v>
@@ -3531,10 +3528,10 @@
         <v>50</v>
       </c>
       <c r="K111" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="O111" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U111" s="1">
         <v>0.35</v>
@@ -3557,10 +3554,10 @@
         <v>50</v>
       </c>
       <c r="O112" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q112" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q112" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="113" spans="1:27">
@@ -3580,16 +3577,16 @@
         <v>50</v>
       </c>
       <c r="O113" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V113" s="1">
         <v>0.35</v>
       </c>
       <c r="W113" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="X113" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="114" spans="1:27">
@@ -3606,25 +3603,25 @@
         <v>51</v>
       </c>
       <c r="F114" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J114" s="1" t="s">
         <v>51</v>
       </c>
       <c r="L114" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N114" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="N114" s="1" t="s">
-        <v>61</v>
-      </c>
       <c r="O114" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P114" s="1">
         <v>5</v>
       </c>
       <c r="Y114" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="115" spans="1:27">
@@ -3641,10 +3638,10 @@
         <v>51</v>
       </c>
       <c r="O115" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z115" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA115" s="1">
         <v>20</v>
@@ -3664,10 +3661,10 @@
         <v>51</v>
       </c>
       <c r="O116" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z116" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA116" s="1">
         <v>20</v>
@@ -3687,10 +3684,10 @@
         <v>51</v>
       </c>
       <c r="O117" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Z117" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AA117" s="1">
         <v>20</v>
@@ -3713,10 +3710,10 @@
         <v>51</v>
       </c>
       <c r="K118" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="O118" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="U118" s="1">
         <v>0.35</v>
@@ -3739,10 +3736,10 @@
         <v>51</v>
       </c>
       <c r="O119" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q119" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="Q119" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="120" spans="1:27">
@@ -3762,198 +3759,16 @@
         <v>51</v>
       </c>
       <c r="O120" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="V120" s="1">
         <v>0.35</v>
       </c>
       <c r="W120" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="X120" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="121" spans="1:27">
-      <c r="A121" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B121" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C121" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D121" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F121" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="J121" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="L121" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="N121" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="O121" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="P121" s="1">
-        <v>5</v>
-      </c>
-      <c r="Y121" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="122" spans="1:27">
-      <c r="A122" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B122" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C122" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D122" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="O122" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="Z122" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="AA122" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="123" spans="1:27">
-      <c r="A123" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B123" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C123" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D123" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="O123" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="Z123" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="AA123" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="124" spans="1:27">
-      <c r="A124" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B124" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C124" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D124" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="O124" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="Z124" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="AA124" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="125" spans="1:27">
-      <c r="A125" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B125" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C125" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D125" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="E125" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="K125" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="O125" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="U125" s="1">
-        <v>0.35</v>
-      </c>
-    </row>
-    <row r="126" spans="1:27">
-      <c r="A126" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B126" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C126" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D126" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="E126" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="O126" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q126" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="127" spans="1:27">
-      <c r="A127" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B127" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C127" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D127" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="E127" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="O127" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="V127" s="1">
-        <v>0.35</v>
-      </c>
-      <c r="W127" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="X127" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>